<commit_message>
Add checklist items for stages 0 and 1
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5UDqLUhrRCiLBZhYj4Swx
</commit_message>
<xml_diff>
--- a/bitrix24-integrator-roadmap.xlsx
+++ b/bitrix24-integrator-roadmap.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Ресурсы и риски" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Чеклист'!$A$1:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Чеклист'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -957,16 +957,16 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Продукт</t>
+          <t>Подготовка</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Настраиваю задачи, шаблоны, Scrum/Канбан</t>
+          <t>Получены права администратора на рабочем портале</t>
         </is>
       </c>
       <c r="D2" s="4">
@@ -983,16 +983,16 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Продукт</t>
+          <t>Подготовка</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Знаю календарь, диск, чат, видеозвонки</t>
+          <t>Выяснен тариф и лимиты (пользователи, диск, роботы, REST)</t>
         </is>
       </c>
       <c r="D3" s="4">
@@ -1009,16 +1009,16 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Подготовка</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Знаю тарифы и ограничения, могу подобрать тариф</t>
+          <t>Создан тестовый портал</t>
         </is>
       </c>
       <c r="D4" s="4">
@@ -1035,16 +1035,16 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Подготовка</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Настраиваю структуру компании и права доступа</t>
+          <t>Заведены аккаунты в Академии и на partners.bitrix24.ru</t>
         </is>
       </c>
       <c r="D5" s="4">
@@ -1061,16 +1061,16 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Подготовка</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Настраиваю рабочие группы, проекты, экстранет</t>
+          <t>Найдены сообщества и чаты интеграторов</t>
         </is>
       </c>
       <c r="D6" s="4">
@@ -1087,16 +1087,16 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Настраиваю безопасность (2FA, IP, журнал)</t>
+          <t>Освоена CRM: лиды, сделки, контакты, компании</t>
         </is>
       </c>
       <c r="D7" s="4">
@@ -1113,16 +1113,16 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Импорт/экспорт данных (CSV, Excel)</t>
+          <t>Освоены открытые линии и контакт-центр</t>
         </is>
       </c>
       <c r="D8" s="4">
@@ -1139,16 +1139,16 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Настроил воронки, стадии, причины отказа</t>
+          <t>Освоены сайты, CRM-формы, онлайн-магазин</t>
         </is>
       </c>
       <c r="D9" s="4">
@@ -1165,16 +1165,16 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Настроил пользовательские поля и справочники</t>
+          <t>Освоены HR, склад, документы/Sign</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -1191,16 +1191,16 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Настроил проверку и объединение дублей</t>
+          <t>Освоены мобильное и десктопное приложения</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -1217,16 +1217,16 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Настроил товары, каталог, счета, КП</t>
+          <t>Освоены отчёты и аналитика</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -1243,16 +1243,16 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Настроил роли и права в CRM</t>
+          <t>Настраиваю задачи, шаблоны, Scrum/Канбан</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -1269,16 +1269,16 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Продукт</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Настроил отчёты, аналитику, дашборды</t>
+          <t>Знаю календарь, диск, чат, видеозвонки</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -1295,16 +1295,16 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Администрирование</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Настроил рассылки и CRM-маркетинг</t>
+          <t>Знаю тарифы и ограничения, могу подобрать тариф</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -1321,16 +1321,16 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>Администрирование</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Роботы и триггеры в лидах и сделках</t>
+          <t>Настраиваю структуру компании и права доступа</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -1347,16 +1347,16 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>Администрирование</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Бизнес-процесс с согласованием</t>
+          <t>Настраиваю рабочие группы, проекты, экстранет</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -1373,16 +1373,16 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>Администрирование</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Смарт-процесс со своими стадиями и полями</t>
+          <t>Настраиваю безопасность (2FA, IP, журнал)</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -1399,16 +1399,16 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>Администрирование</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Шаблоны документов и генерация из CRM</t>
+          <t>Импорт/экспорт данных (CSV, Excel)</t>
         </is>
       </c>
       <c r="D19" s="4">
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>SLA и эскалации</t>
+          <t>Настроил воронки, стадии, причины отказа</t>
         </is>
       </c>
       <c r="D20" s="4">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Автоматизация</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Шаблоны БП для Живой ленты (заявка, отпуск, командировка)</t>
+          <t>Настроил пользовательские поля и справочники</t>
         </is>
       </c>
       <c r="D21" s="4">
@@ -1477,16 +1477,16 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Подключил почту и календарь</t>
+          <t>Настроил проверку и объединение дублей</t>
         </is>
       </c>
       <c r="D22" s="4">
@@ -1503,16 +1503,16 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Подключил телефонию и записи звонков</t>
+          <t>Настроил товары, каталог, счета, КП</t>
         </is>
       </c>
       <c r="D23" s="4">
@@ -1529,16 +1529,16 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Подключил открытые линии (мессенджеры, сайт)</t>
+          <t>Настроил роли и права в CRM</t>
         </is>
       </c>
       <c r="D24" s="4">
@@ -1555,16 +1555,16 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>CRM-формы и передача UTM / сквозная аналитика</t>
+          <t>Настроил отчёты, аналитику, дашборды</t>
         </is>
       </c>
       <c r="D25" s="4">
@@ -1581,16 +1581,16 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Знаю варианты интеграции с 1С и умею выбирать</t>
+          <t>Настроил рассылки и CRM-маркетинг</t>
         </is>
       </c>
       <c r="D26" s="4">
@@ -1607,16 +1607,16 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Связка сервисов через Make/n8n</t>
+          <t>Роботы и триггеры в лидах и сделках</t>
         </is>
       </c>
       <c r="D27" s="4">
@@ -1633,16 +1633,16 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Интеграции</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Умею оценивать приложения Маркета</t>
+          <t>Бизнес-процесс с согласованием</t>
         </is>
       </c>
       <c r="D28" s="4">
@@ -1659,16 +1659,16 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Вызов REST через входящий вебхук (crm.lead.add, crm.deal.list)</t>
+          <t>Смарт-процесс со своими стадиями и полями</t>
         </is>
       </c>
       <c r="D29" s="4">
@@ -1685,16 +1685,16 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Исходящий вебхук и обработка события</t>
+          <t>Шаблоны документов и генерация из CRM</t>
         </is>
       </c>
       <c r="D30" s="4">
@@ -1711,16 +1711,16 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Локальное приложение с OAuth</t>
+          <t>SLA и эскалации</t>
         </is>
       </c>
       <c r="D31" s="4">
@@ -1737,16 +1737,16 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Автоматизация</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Использую batch и учитываю лимиты</t>
+          <t>Шаблоны БП для Живой ленты (заявка, отпуск, командировка)</t>
         </is>
       </c>
       <c r="D32" s="4">
@@ -1763,16 +1763,16 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Собственный робот/активити для БП</t>
+          <t>Подключил почту и календарь</t>
         </is>
       </c>
       <c r="D33" s="4">
@@ -1789,16 +1789,16 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Встройка (placement) в интерфейс</t>
+          <t>Подключил телефонию и записи звонков</t>
         </is>
       </c>
       <c r="D34" s="4">
@@ -1815,16 +1815,16 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Отладка, логирование, безопасное хранение токенов</t>
+          <t>Подключил открытые линии (мессенджеры, сайт)</t>
         </is>
       </c>
       <c r="D35" s="4">
@@ -1841,16 +1841,16 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Разработка</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Развёртывание приложения по HTTPS</t>
+          <t>CRM-формы и передача UTM / сквозная аналитика</t>
         </is>
       </c>
       <c r="D36" s="4">
@@ -1867,16 +1867,16 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Обследование и описание процессов</t>
+          <t>Знаю варианты интеграции с 1С и умею выбирать</t>
         </is>
       </c>
       <c r="D37" s="4">
@@ -1893,16 +1893,16 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>ТЗ и оценка сроков</t>
+          <t>Связка сервисов через Make/n8n</t>
         </is>
       </c>
       <c r="D38" s="4">
@@ -1919,16 +1919,16 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Интеграции</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Обучение и инструкции для пользователей</t>
+          <t>Умею оценивать приложения Маркета</t>
         </is>
       </c>
       <c r="D39" s="4">
@@ -1945,16 +1945,16 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Ведение проекта: этапы, риски, приёмка</t>
+          <t>Вызов REST через входящий вебхук (crm.lead.add, crm.deal.list)</t>
         </is>
       </c>
       <c r="D40" s="4">
@@ -1971,16 +1971,16 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Договор, SLA, порядок поддержки</t>
+          <t>Исходящий вебхук и обработка события</t>
         </is>
       </c>
       <c r="D41" s="4">
@@ -1997,16 +1997,16 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Методология</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Расчёт окупаемости внедрения</t>
+          <t>Локальное приложение с OAuth</t>
         </is>
       </c>
       <c r="D42" s="4">
@@ -2023,16 +2023,16 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Пройдено обучение в Академии Битрикс24</t>
+          <t>Использую batch и учитываю лимиты</t>
         </is>
       </c>
       <c r="D43" s="4">
@@ -2049,16 +2049,16 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Получены сертификаты</t>
+          <t>Собственный робот/активити для БП</t>
         </is>
       </c>
       <c r="D44" s="4">
@@ -2075,16 +2075,16 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>≥3 кейса на внутреннем портале</t>
+          <t>Встройка (placement) в интерфейс</t>
         </is>
       </c>
       <c r="D45" s="4">
@@ -2101,16 +2101,16 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Портфолио и отзывы</t>
+          <t>Отладка, логирование, безопасное хранение токенов</t>
         </is>
       </c>
       <c r="D46" s="4">
@@ -2127,16 +2127,16 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Разработка</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Статус партнёра (если целесообразно)</t>
+          <t>Развёртывание приложения по HTTPS</t>
         </is>
       </c>
       <c r="D47" s="4">
@@ -2153,16 +2153,16 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Методология</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Первый внешний клиент</t>
+          <t>Обследование и описание процессов</t>
         </is>
       </c>
       <c r="D48" s="4">
@@ -2177,16 +2177,302 @@
       <c r="F48" s="9" t="n"/>
       <c r="G48" s="4" t="n"/>
     </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>ТЗ и оценка сроков</t>
+        </is>
+      </c>
+      <c r="D49" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A49,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="4" t="n"/>
+    </row>
     <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="A50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Обучение и инструкции для пользователей</t>
+        </is>
+      </c>
+      <c r="D50" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A50,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Ведение проекта: этапы, риски, приёмка</t>
+        </is>
+      </c>
+      <c r="D51" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A51,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n"/>
+      <c r="G51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Договор, SLA, порядок поддержки</t>
+        </is>
+      </c>
+      <c r="D52" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A52,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Методология</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Расчёт окупаемости внедрения</t>
+        </is>
+      </c>
+      <c r="D53" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A53,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Пройдено обучение в Академии Битрикс24</t>
+        </is>
+      </c>
+      <c r="D54" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A54,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n"/>
+      <c r="G54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Получены сертификаты</t>
+        </is>
+      </c>
+      <c r="D55" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A55,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n"/>
+      <c r="G55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>≥3 кейса на внутреннем портале</t>
+        </is>
+      </c>
+      <c r="D56" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A56,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n"/>
+      <c r="G56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Портфолио и отзывы</t>
+        </is>
+      </c>
+      <c r="D57" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A57,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n"/>
+      <c r="G57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Статус партнёра (если целесообразно)</t>
+        </is>
+      </c>
+      <c r="D58" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A58,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n"/>
+      <c r="G58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Первый внешний клиент</t>
+        </is>
+      </c>
+      <c r="D59" s="4">
+        <f>INDEX('Дорожная карта'!$B$5:$B$12,MATCH(A59,'Дорожная карта'!$A$5:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n"/>
+      <c r="G59" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>Легенда: меняйте только синие ячейки в колонке «Статус» (выпадающий список), дату и заметки.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G48"/>
-  <conditionalFormatting sqref="E2:E48">
+  <autoFilter ref="A1:G59"/>
+  <conditionalFormatting sqref="E2:E59">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Готово"</formula>
     </cfRule>
@@ -2195,7 +2481,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Не начато,В работе,Готово"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>